<commit_message>
Extra rows removed from Fabrication BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Fabrication BOM .xlsx
+++ b/Deliverables/BOM/Fabrication BOM .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SaleemD-CustomProduct\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E04563-3EA6-4B2E-8F05-CA16B1888CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5232C4B5-3182-404E-B6C5-108EF25ECFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>S. No.</t>
   </si>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t>LCSC/MOQ</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>C194427</t>
@@ -356,7 +353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -414,16 +411,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -706,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="5" bestFit="1" customWidth="1"/>
@@ -715,11 +709,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="A1" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
     </row>
     <row r="2" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
@@ -737,7 +731,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" s="15">
         <v>10</v>
@@ -750,7 +744,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" s="11">
         <v>7</v>
@@ -763,7 +757,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" s="11">
         <v>50</v>
@@ -776,7 +770,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="11">
         <v>100</v>
@@ -789,7 +783,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" s="11">
         <v>100</v>
@@ -802,7 +796,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="11">
         <v>20</v>
@@ -815,7 +809,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" s="11">
         <v>50</v>
@@ -828,7 +822,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="11">
         <v>20</v>
@@ -841,7 +835,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="11">
         <v>100</v>
@@ -854,7 +848,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="12">
         <v>50</v>
@@ -867,7 +861,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="15">
         <v>40</v>
@@ -880,7 +874,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" s="12">
         <v>12</v>
@@ -893,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15" s="19">
         <v>7</v>
@@ -906,7 +900,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C16" s="17">
         <v>20</v>
@@ -919,7 +913,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C17" s="15">
         <v>50</v>
@@ -932,7 +926,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="11">
         <v>10</v>
@@ -945,7 +939,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="11">
         <v>100</v>
@@ -958,7 +952,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="11">
         <v>100</v>
@@ -971,7 +965,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" s="11">
         <v>40</v>
@@ -984,7 +978,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C22" s="11">
         <v>100</v>
@@ -997,7 +991,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C23" s="11">
         <v>50</v>
@@ -1010,7 +1004,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="3">
         <v>100</v>
@@ -1023,7 +1017,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C25" s="4">
         <v>100</v>
@@ -1035,8 +1029,8 @@
       <c r="A26" s="8">
         <v>24</v>
       </c>
-      <c r="B26" s="23" t="s">
-        <v>33</v>
+      <c r="B26" s="21" t="s">
+        <v>32</v>
       </c>
       <c r="C26" s="1">
         <v>12</v>
@@ -1049,7 +1043,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" s="4">
         <v>7</v>
@@ -1059,12 +1053,12 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
-        <v>26</v>
-      </c>
-      <c r="B28" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="C28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="4">
         <v>7</v>
       </c>
       <c r="D28" s="2"/>
@@ -1072,25 +1066,25 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="8">
-        <v>27</v>
-      </c>
-      <c r="B29" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C29" s="4">
-        <v>7</v>
+      <c r="C29" s="1">
+        <v>6</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8">
-        <v>28</v>
-      </c>
-      <c r="B30" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="11">
         <v>6</v>
       </c>
       <c r="D30" s="2"/>
@@ -1098,23 +1092,23 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
-        <v>29</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>3</v>
+        <v>31</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="C31" s="11">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
     </row>
     <row r="32" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C32" s="11">
         <v>6</v>
@@ -1124,104 +1118,77 @@
     </row>
     <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
-        <v>31</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C33" s="11">
-        <v>25</v>
+        <v>34</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="15">
+        <v>30</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
     </row>
     <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C34" s="11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
     </row>
     <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8">
-        <v>33</v>
-      </c>
-      <c r="B35" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="C35" s="12">
-        <v>30</v>
+        <v>36</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C35" s="11">
+        <v>7</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
     <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="8">
-        <v>34</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="15">
-        <v>30</v>
+        <v>37</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="12">
+        <v>7</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8">
-        <v>35</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C37" s="11">
-        <v>7</v>
-      </c>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8">
-        <v>36</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C38" s="11">
-        <v>7</v>
-      </c>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="8">
-        <v>37</v>
-      </c>
-      <c r="B39" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" s="12">
-        <v>7</v>
-      </c>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
     </row>
@@ -1269,7 +1236,7 @@
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
     </row>
@@ -1281,7 +1248,7 @@
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="4:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
     </row>
@@ -1292,18 +1259,6 @@
     <row r="58" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
-    </row>
-    <row r="59" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-    </row>
-    <row r="60" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-    </row>
-    <row r="61" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>